<commit_message>
Fix incorrect scores in the excel files
</commit_message>
<xml_diff>
--- a/Notas_da_Copa_2026.xlsx
+++ b/Notas_da_Copa_2026.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="204">
   <si>
     <t>Controle de notas — Copa do Mundo 2026</t>
   </si>
@@ -633,6 +633,9 @@
   </si>
   <si>
     <t>Espanha x Argentina</t>
+  </si>
+  <si>
+    <t>2-3</t>
   </si>
 </sst>
 </file>
@@ -9251,7 +9254,7 @@
         <v>188</v>
       </c>
       <c r="E6" s="32" t="s">
-        <v>125</v>
+        <v>203</v>
       </c>
       <c r="F6" s="36">
         <v>7.0</v>

</xml_diff>